<commit_message>
Refresh live data 2026-09-07T16:33Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-04T15:00:44Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-07T16:33:05Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-04T15:00:44Z</t>
+          <t>Last refreshed: 2026-09-07T16:33:05Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.79</v>
+        <v>4.77</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.43</v>
+        <v>0.41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.757</v>
+        <v>17.19</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-04T15:00:44Z</t>
+          <t>2026-09-07T16:33:05Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.7699890136719</v>
+        <v>285.739990234375</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.70000076293945</v>
+        <v>43.72999954223633</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>62.43999862670898</v>
+        <v>63.29000091552734</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>606.2449951171875</v>
+        <v>604.719970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>219.2050018310547</v>
+        <v>219.6000061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-08T15:11Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-07T16:33:05Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-08T15:11:24Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-07T16:33:05Z</t>
+          <t>Last refreshed: 2026-09-08T15:11:24Z</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32346,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32438,7 +32438,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-07T16:33:05Z</t>
+          <t>2026-09-08T15:11:24Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.739990234375</v>
+        <v>285.9800109863281</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>43.72999954223633</v>
+        <v>42.77000045776367</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>63.29000091552734</v>
+        <v>60.88999938964844</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>604.719970703125</v>
+        <v>600.594970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>219.6000061035156</v>
+        <v>216.0549926757812</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-09T15:11Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-08T15:11:24Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-09T15:11:15Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-08T15:11:24Z</t>
+          <t>Last refreshed: 2026-09-09T15:11:15Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.77</v>
+        <v>4.78</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-08T15:11:24Z</t>
+          <t>2026-09-09T15:11:15Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.9800109863281</v>
+        <v>281.5400085449219</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.77000045776367</v>
+        <v>41.97000122070312</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>60.88999938964844</v>
+        <v>60.29999923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>600.594970703125</v>
+        <v>592.2100219726562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>216.0549926757812</v>
+        <v>212.8699951171875</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-10T15:03Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-09T15:11:15Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-10T15:03:13Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-09T15:11:15Z</t>
+          <t>Last refreshed: 2026-09-10T15:03:13Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.78</v>
+        <v>4.8</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32392,7 +32392,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-09T15:11:15Z</t>
+          <t>2026-09-10T15:03:13Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.5400085449219</v>
+        <v>279.7157897949219</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>41.97000122070312</v>
+        <v>41.75</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>60.29999923706055</v>
+        <v>60.65000152587891</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>592.2100219726562</v>
+        <v>599.760009765625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>212.8699951171875</v>
+        <v>206.5399932861328</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-11T15:06Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-10T15:03:13Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-11T15:06:04Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-10T15:03:13Z</t>
+          <t>Last refreshed: 2026-09-11T15:06:04Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.8</v>
+        <v>4.83</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32501,7 +32501,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>184.661</v>
+        <v>184.58</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -32525,12 +32525,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.71</v>
+        <v>6.76</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-10T15:03:13Z</t>
+          <t>2026-09-11T15:06:04Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>279.7157897949219</v>
+        <v>281.239990234375</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>41.75</v>
+        <v>41.68500137329102</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>60.65000152587891</v>
+        <v>62.20000076293945</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>599.760009765625</v>
+        <v>604.5700073242188</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>206.5399932861328</v>
+        <v>207.6499938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-14T16:59Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-11T15:06:04Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-14T16:59:00Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-11T15:06:04Z</t>
+          <t>Last refreshed: 2026-09-14T16:59:00Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.83</v>
+        <v>4.95</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-11T15:06:04Z</t>
+          <t>2026-09-14T16:59:00Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.239990234375</v>
+        <v>283.5549926757812</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>41.68500137329102</v>
+        <v>42.27500152587891</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>62.20000076293945</v>
+        <v>61.70999908447266</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>604.5700073242188</v>
+        <v>605.157470703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>207.6499938964844</v>
+        <v>208.1399993896484</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-15T15:36Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-14T16:59:00Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-15T15:36:43Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-14T16:59:00Z</t>
+          <t>Last refreshed: 2026-09-15T15:36:43Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.95</v>
+        <v>4.96</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-14T16:59:00Z</t>
+          <t>2026-09-15T15:36:43Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>283.5549926757812</v>
+        <v>282.7099914550781</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>42.27500152587891</v>
+        <v>40.72499847412109</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>61.70999908447266</v>
+        <v>60.34000015258789</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>605.157470703125</v>
+        <v>590.5900268554688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>208.1399993896484</v>
+        <v>203.9049987792969</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-16T15:27Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-15T15:36:43Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-16T15:26:55Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-15T15:36:43Z</t>
+          <t>Last refreshed: 2026-09-16T15:26:55Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.96</v>
+        <v>4.97</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-15T15:36:43Z</t>
+          <t>2026-09-16T15:26:55Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>282.7099914550781</v>
+        <v>286.2799987792969</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>40.72499847412109</v>
+        <v>41.22999954223633</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>60.34000015258789</v>
+        <v>59.56999969482422</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>590.5900268554688</v>
+        <v>602.9400024414062</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>203.9049987792969</v>
+        <v>207.1000061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-17T15:34Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-16T15:26:55Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-17T15:34:38Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-16T15:26:55Z</t>
+          <t>Last refreshed: 2026-09-17T15:34:38Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.97</v>
+        <v>5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32392,7 +32392,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.33</v>
+        <v>0.27</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-16T15:26:55Z</t>
+          <t>2026-09-17T15:34:38Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>286.2799987792969</v>
+        <v>284.8399963378906</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>41.22999954223633</v>
+        <v>40.81999969482422</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>59.56999969482422</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>602.9400024414062</v>
+        <v>592.8350219726562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>207.1000061035156</v>
+        <v>203.7700042724609</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-18T15:03Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-17T15:34:38Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-18T15:03:03Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-17T15:34:38Z</t>
+          <t>Last refreshed: 2026-09-18T15:03:03Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>5.01</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32363,7 +32363,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.76</v>
+        <v>6.95</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-17T15:34:38Z</t>
+          <t>2026-09-18T15:03:03Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>284.8399963378906</v>
+        <v>281.5199890136719</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>40.81999969482422</v>
+        <v>40.11999893188477</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.5</v>
+        <v>58.83499908447266</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>592.8350219726562</v>
+        <v>577.1199951171875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>203.7700042724609</v>
+        <v>201.8099975585938</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-21T17:07Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-18T15:03:03Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-21T17:07:08Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-18T15:03:03Z</t>
+          <t>Last refreshed: 2026-09-21T17:07:08Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.01</v>
+        <v>4.94</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.27</v>
+        <v>0.25</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-18T15:03:03Z</t>
+          <t>2026-09-21T17:07:08Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.5199890136719</v>
+        <v>280.4800109863281</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>40.11999893188477</v>
+        <v>40.04000091552734</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.83499908447266</v>
+        <v>58.40499877929688</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>577.1199951171875</v>
+        <v>581.4550170898438</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>201.8099975585938</v>
+        <v>204.4499969482422</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-22T15:33Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-21T17:07:08Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-22T15:33:02Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-21T17:07:08Z</t>
+          <t>Last refreshed: 2026-09-22T15:33:02Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.94</v>
+        <v>5.01</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-21T17:07:08Z</t>
+          <t>2026-09-22T15:33:02Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>280.4800109863281</v>
+        <v>274.9200134277344</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>40.04000091552734</v>
+        <v>39.46500015258789</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.40499877929688</v>
+        <v>56.91999816894531</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>581.4550170898438</v>
+        <v>552.989990234375</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.4499969482422</v>
+        <v>200.1049957275391</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-23T15:28Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-22T15:33:02Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-23T15:28:50Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-22T15:33:02Z</t>
+          <t>Last refreshed: 2026-09-23T15:28:50Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.01</v>
+        <v>4.96</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-22T15:33:02Z</t>
+          <t>2026-09-23T15:28:50Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>274.9200134277344</v>
+        <v>271.6998901367188</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>39.46500015258789</v>
+        <v>38.77000045776367</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>56.91999816894531</v>
+        <v>56.83000183105469</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>552.989990234375</v>
+        <v>548.8049926757812</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>200.1049957275391</v>
+        <v>197.4900054931641</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-24T15:51Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-23T15:28:50Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-24T15:51:08Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-23T15:28:50Z</t>
+          <t>Last refreshed: 2026-09-24T15:51:08Z</t>
         </is>
       </c>
     </row>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-23T15:28:50Z</t>
+          <t>2026-09-24T15:51:08Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>271.6998901367188</v>
+        <v>264.4049987792969</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.77000045776367</v>
+        <v>38.28499984741211</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>56.83000183105469</v>
+        <v>55.95000076293945</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>548.8049926757812</v>
+        <v>546.9600219726562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>197.4900054931641</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-25T15:51Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-24T15:51:08Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-25T15:51:26Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-24T15:51:08Z</t>
+          <t>Last refreshed: 2026-09-25T15:51:26Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.96</v>
+        <v>5.11</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.26</v>
+        <v>0.31</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>55.2</v>
+        <v>51.7</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.95</v>
+        <v>7.03</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-24T15:51:08Z</t>
+          <t>2026-09-25T15:51:26Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>264.4049987792969</v>
+        <v>265.2000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.28499984741211</v>
+        <v>38.47000122070312</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>55.95000076293945</v>
+        <v>56.47499847412109</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>546.9600219726562</v>
+        <v>553</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>195</v>
+        <v>197.8099975585938</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-28T18:38Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-25T15:51:26Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-28T18:38:45Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-25T15:51:26Z</t>
+          <t>Last refreshed: 2026-09-28T18:38:45Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.11</v>
+        <v>5.18</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-25T15:51:26Z</t>
+          <t>2026-09-28T18:38:45Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>265.2000122070312</v>
+        <v>264.0799865722656</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.47000122070312</v>
+        <v>38.30500030517578</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>56.47499847412109</v>
+        <v>56.97000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>553</v>
+        <v>546.4099731445312</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>197.8099975585938</v>
+        <v>197.6499938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-29T16:55Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-28T18:38:45Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-29T16:55:23Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-28T18:38:45Z</t>
+          <t>Last refreshed: 2026-09-29T16:55:23Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.18</v>
+        <v>5.17</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-28T18:38:45Z</t>
+          <t>2026-09-29T16:55:23Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>264.0799865722656</v>
+        <v>261.7799987792969</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.30500030517578</v>
+        <v>37.63999938964844</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>56.97000122070312</v>
+        <v>58.99750137329102</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>546.4099731445312</v>
+        <v>536.2150268554688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>197.6499938964844</v>
+        <v>196.4349975585938</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-09-30T16:52Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-29T16:55:23Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-09-30T16:52:25Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-29T16:55:23Z</t>
+          <t>Last refreshed: 2026-09-30T16:52:25Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.17</v>
+        <v>5.24</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17.19</v>
+        <v>16.982</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32731,7 +32731,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>207.457</v>
+        <v>187.097</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -32755,12 +32755,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-29T16:55:23Z</t>
+          <t>2026-09-30T16:52:25Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>261.7799987792969</v>
+        <v>263.4800109863281</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.63999938964844</v>
+        <v>37.22999954223633</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>58.99750137329102</v>
+        <v>56.70000076293945</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>536.2150268554688</v>
+        <v>530.4249877929688</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>196.4349975585938</v>
+        <v>193.8099975585938</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-01T17:25Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-09-30T16:52:25Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-01T17:25:16Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-09-30T16:52:25Z</t>
+          <t>Last refreshed: 2026-10-01T17:25:16Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.24</v>
+        <v>5.26</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.37</v>
+        <v>0.41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7.03</v>
+        <v>7.28</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-09-30T16:52:25Z</t>
+          <t>2026-10-01T17:25:16Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>263.4800109863281</v>
+        <v>266.4800109863281</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.22999954223633</v>
+        <v>37.27000045776367</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>56.70000076293945</v>
+        <v>55.72000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>530.4249877929688</v>
+        <v>513.02001953125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>193.8099975585938</v>
+        <v>193.2299957275391</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-02T16:43Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-01T17:25:16Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-02T16:43:05Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-01T17:25:16Z</t>
+          <t>Last refreshed: 2026-10-02T16:43:05Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.26</v>
+        <v>5.29</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.41</v>
+        <v>0.46</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32593,7 +32593,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -32617,12 +32617,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-01T17:25:16Z</t>
+          <t>2026-10-02T16:43:05Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>266.4800109863281</v>
+        <v>266.5899963378906</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.27000045776367</v>
+        <v>38.09999847412109</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>55.72000122070312</v>
+        <v>54.77000045776367</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>513.02001953125</v>
+        <v>527.844970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>193.2299957275391</v>
+        <v>195.0099945068359</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-06T17:18Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-02T16:43:05Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-06T17:18:12Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-02T16:43:05Z</t>
+          <t>Last refreshed: 2026-10-06T17:18:12Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.29</v>
+        <v>5.28</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.982</v>
+        <v>16.378</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-02T16:43:05Z</t>
+          <t>2026-10-06T17:18:12Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>266.5899963378906</v>
+        <v>268.3999938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.09999847412109</v>
+        <v>37.66999816894531</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>54.77000045776367</v>
+        <v>55.4119987487793</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>527.844970703125</v>
+        <v>538.0601196289062</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>195.0099945068359</v>
+        <v>196</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-07T17:51Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-06T17:18:12Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-07T17:51:36Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-06T17:18:12Z</t>
+          <t>Last refreshed: 2026-10-07T17:51:36Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.28</v>
+        <v>5.31</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.47</v>
+        <v>0.48</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-06T17:18:12Z</t>
+          <t>2026-10-07T17:51:36Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>268.3999938964844</v>
+        <v>269.1700134277344</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.66999816894531</v>
+        <v>37.36999893188477</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>55.4119987487793</v>
+        <v>53.29999923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>538.0601196289062</v>
+        <v>535.75</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>196</v>
+        <v>195.3999938964844</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-08T17:55Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-07T17:51:36Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-08T17:55:09Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-07T17:51:36Z</t>
+          <t>Last refreshed: 2026-10-08T17:55:09Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.31</v>
+        <v>5.27</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.48</v>
+        <v>0.51</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7.28</v>
+        <v>7.4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32685,7 +32685,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>297771</v>
+        <v>294124</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -32709,12 +32709,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32801,12 +32801,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-07T17:51:36Z</t>
+          <t>2026-10-08T17:55:09Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>269.1700134277344</v>
+        <v>272.9500122070312</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.36999893188477</v>
+        <v>37.52999877929688</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.29999923706055</v>
+        <v>53.6150016784668</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>535.75</v>
+        <v>540.219970703125</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>195.3999938964844</v>
+        <v>196.0899963378906</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-09T17:28Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-08T17:55:09Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-09T17:28:38Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-08T17:55:09Z</t>
+          <t>Last refreshed: 2026-10-09T17:28:38Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.27</v>
+        <v>5.28</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.51</v>
+        <v>0.47</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-08T17:55:09Z</t>
+          <t>2026-10-09T17:28:38Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>272.9500122070312</v>
+        <v>267.7550048828125</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.52999877929688</v>
+        <v>37.46500015258789</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.6150016784668</v>
+        <v>52.72000122070312</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>540.219970703125</v>
+        <v>538.4199829101562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>196.0899963378906</v>
+        <v>199.6100006103516</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-12T20:20Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-09T17:28:38Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-12T20:20:49Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-09T17:28:38Z</t>
+          <t>Last refreshed: 2026-10-12T20:20:49Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.28</v>
+        <v>5.22</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.47</v>
+        <v>0.44</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-09T17:28:38Z</t>
+          <t>2026-10-12T20:20:49Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>267.7550048828125</v>
+        <v>268.6300048828125</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.46500015258789</v>
+        <v>37.90999984741211</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.72000122070312</v>
+        <v>50.68999862670898</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>538.4199829101562</v>
+        <v>548.1199951171875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>199.6100006103516</v>
+        <v>201.1399993896484</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-13T18:23Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-12T20:20:49Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-13T18:23:24Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-12T20:20:49Z</t>
+          <t>Last refreshed: 2026-10-13T18:23:24Z</t>
         </is>
       </c>
     </row>
@@ -32346,7 +32346,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32438,7 +32438,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-12T20:20:49Z</t>
+          <t>2026-10-13T18:23:24Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>268.6300048828125</v>
+        <v>270.4700012207031</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.90999984741211</v>
+        <v>37.54499816894531</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>50.68999862670898</v>
+        <v>50.46500015258789</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>548.1199951171875</v>
+        <v>543.9199829101562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>201.1399993896484</v>
+        <v>196.5700073242188</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-14T15:52Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-13T18:23:24Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-14T15:52:02Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-13T18:23:24Z</t>
+          <t>Last refreshed: 2026-10-14T15:52:02Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.22</v>
+        <v>5.24</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.44</v>
+        <v>0.42</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32501,7 +32501,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>184.58</v>
+        <v>184.395</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -32525,12 +32525,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-13T18:23:24Z</t>
+          <t>2026-10-14T15:52:02Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>270.4700012207031</v>
+        <v>272.3500061035156</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.54499816894531</v>
+        <v>36.72969818115234</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>50.46500015258789</v>
+        <v>49.34999847412109</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>543.9199829101562</v>
+        <v>533.2249755859375</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>196.5700073242188</v>
+        <v>195.2599945068359</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-15T15:38Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-14T15:52:02Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-15T15:38:46Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-14T15:52:02Z</t>
+          <t>Last refreshed: 2026-10-15T15:38:46Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.24</v>
+        <v>5.21</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.42</v>
+        <v>0.37</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-14T15:52:02Z</t>
+          <t>2026-10-15T15:38:46Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>272.3500061035156</v>
+        <v>280.5650024414062</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>36.72969818115234</v>
+        <v>37.59000015258789</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>49.34999847412109</v>
+        <v>51.91999816894531</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>533.2249755859375</v>
+        <v>545.6799926757812</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>195.2599945068359</v>
+        <v>196.3399963378906</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-16T15:24Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-15T15:38:46Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-16T15:24:32Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-15T15:38:46Z</t>
+          <t>Last refreshed: 2026-10-16T15:24:32Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.21</v>
+        <v>5.19</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-15T15:38:46Z</t>
+          <t>2026-10-16T15:24:32Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>280.5650024414062</v>
+        <v>285.2999877929688</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.59000015258789</v>
+        <v>38.20000076293945</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>51.91999816894531</v>
+        <v>54.22999954223633</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>545.6799926757812</v>
+        <v>549.280029296875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>196.3399963378906</v>
+        <v>202.8500061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-19T17:35Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-16T15:24:32Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-19T17:35:32Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-16T15:24:32Z</t>
+          <t>Last refreshed: 2026-10-19T17:35:32Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.19</v>
+        <v>5.1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-16T15:24:32Z</t>
+          <t>2026-10-19T17:35:32Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.2999877929688</v>
+        <v>281.6600036621094</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.20000076293945</v>
+        <v>37.45500183105469</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>54.22999954223633</v>
+        <v>52.16999816894531</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>549.280029296875</v>
+        <v>539.4151000976562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>202.8500061035156</v>
+        <v>199.6000061035156</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-20T15:41Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-19T17:35:32Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-20T15:41:29Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-19T17:35:32Z</t>
+          <t>Last refreshed: 2026-10-20T15:41:29Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.1</v>
+        <v>5.09</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-19T17:35:32Z</t>
+          <t>2026-10-20T15:41:29Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>281.6600036621094</v>
+        <v>285.25</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.45500183105469</v>
+        <v>37.93999862670898</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>52.16999816894531</v>
+        <v>53.25</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>539.4151000976562</v>
+        <v>539.6599731445312</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>199.6000061035156</v>
+        <v>202.0200042724609</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-21T15:59Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-20T15:41:29Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-21T15:59:47Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-20T15:41:29Z</t>
+          <t>Last refreshed: 2026-10-21T15:59:47Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.09</v>
+        <v>400</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32363,7 +32363,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>400</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.38</v>
+        <v>400</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16.378</v>
+        <v>400</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32501,7 +32501,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>184.395</v>
+        <v>400</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -32525,12 +32525,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>51.7</v>
+        <v>400</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32593,7 +32593,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4.2</v>
+        <v>400</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -32617,12 +32617,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7.4</v>
+        <v>400</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32685,7 +32685,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>294124</v>
+        <v>400</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -32709,12 +32709,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32731,7 +32731,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>187.097</v>
+        <v>400</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -32755,12 +32755,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32777,7 +32777,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7.47</v>
+        <v>400</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -32801,12 +32801,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-20T15:41:29Z</t>
+          <t>2026-10-21T15:59:47Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.25</v>
+        <v>284.8150024414062</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>37.93999862670898</v>
+        <v>38.61920166015625</v>
       </c>
     </row>
     <row r="20">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>539.6599731445312</v>
+        <v>539.3424072265625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>202.0200042724609</v>
+        <v>210.1300048828125</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-22T15:55Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-21T15:59:47Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-22T15:55:31Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-21T15:59:47Z</t>
+          <t>Last refreshed: 2026-10-22T15:55:31Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>400</v>
+        <v>5.12</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32363,7 +32363,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>400</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>400</v>
+        <v>0.32</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32455,7 +32455,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>400</v>
+        <v>16.378</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -32479,12 +32479,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32501,7 +32501,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>400</v>
+        <v>184.395</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -32525,12 +32525,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>400</v>
+        <v>51.7</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32593,7 +32593,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>400</v>
+        <v>4.2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -32617,12 +32617,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>400</v>
+        <v>7.4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32685,7 +32685,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>400</v>
+        <v>294124</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -32709,12 +32709,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32731,7 +32731,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>400</v>
+        <v>187.097</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -32755,12 +32755,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32777,7 +32777,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>400</v>
+        <v>7.47</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -32801,12 +32801,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    &lt;link href="https://fonts.googleapis.com/css?family=Open+Sans:300</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-21T15:59:47Z</t>
+          <t>2026-10-22T15:55:31Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>284.8150024414062</v>
+        <v>287.125</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.61920166015625</v>
+        <v>38.75249862670898</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.25</v>
+        <v>51.87099838256836</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>539.3424072265625</v>
+        <v>548.7852172851562</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>210.1300048828125</v>
+        <v>204.5899963378906</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-23T15:47Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-22T15:55:31Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-23T15:47:32Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-22T15:55:31Z</t>
+          <t>Last refreshed: 2026-10-23T15:47:32Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.12</v>
+        <v>5.13</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32547,7 +32547,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>51.7</v>
+        <v>48.1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -32571,12 +32571,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7.4</v>
+        <v>7.32</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-22T15:55:31Z</t>
+          <t>2026-10-23T15:47:32Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>287.125</v>
+        <v>285.177490234375</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.75249862670898</v>
+        <v>39.02000045776367</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>51.87099838256836</v>
+        <v>50.92499923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>548.7852172851562</v>
+        <v>546.655029296875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.5899963378906</v>
+        <v>201.0399932861328</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-26T17:29Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-23T15:47:32Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-26T17:28:56Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-23T15:47:32Z</t>
+          <t>Last refreshed: 2026-10-26T17:28:56Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5.13</v>
+        <v>4.96</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-23T15:47:32Z</t>
+          <t>2026-10-26T17:28:56Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.177490234375</v>
+        <v>287.3699951171875</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>39.02000045776367</v>
+        <v>38.91500091552734</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>50.92499923706055</v>
+        <v>53.29499816894531</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>546.655029296875</v>
+        <v>541.5599975585938</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>201.0399932861328</v>
+        <v>202.8699951171875</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-27T16:44Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-26T17:28:56Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-27T16:44:18Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-26T17:28:56Z</t>
+          <t>Last refreshed: 2026-10-27T16:44:18Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.96</v>
+        <v>5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-26T17:28:56Z</t>
+          <t>2026-10-27T16:44:18Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>287.3699951171875</v>
+        <v>285.3250122070312</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.91500091552734</v>
+        <v>39.06999969482422</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.29499816894531</v>
+        <v>53.95500183105469</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>541.5599975585938</v>
+        <v>540.4000244140625</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>202.8699951171875</v>
+        <v>204.1300048828125</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-28T17:12Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-27T16:44:18Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-28T17:12:44Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-27T16:44:18Z</t>
+          <t>Last refreshed: 2026-10-28T17:12:44Z</t>
         </is>
       </c>
     </row>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.32</v>
+        <v>0.29</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-27T16:44:18Z</t>
+          <t>2026-10-28T17:12:44Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.3250122070312</v>
+        <v>285.625</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>39.06999969482422</v>
+        <v>38.74200057983398</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.95500183105469</v>
+        <v>53.54999923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>540.4000244140625</v>
+        <v>542.4400024414062</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.1300048828125</v>
+        <v>204.2949981689453</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-29T17:28Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-28T17:12:44Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-29T17:28:08Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-28T17:12:44Z</t>
+          <t>Last refreshed: 2026-10-29T17:28:08Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>4.99</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.29</v>
+        <v>0.38</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32639,7 +32639,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7.32</v>
+        <v>7.24</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -32663,12 +32663,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-28T17:12:44Z</t>
+          <t>2026-10-29T17:28:08Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>285.625</v>
+        <v>291.2749938964844</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>38.74200057983398</v>
+        <v>39.70000076293945</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>53.54999923706055</v>
+        <v>55.42499923706055</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>542.4400024414062</v>
+        <v>564.1199951171875</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>204.2949981689453</v>
+        <v>208.7449951171875</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>

<commit_message>
Refresh live data 2026-10-30T17:03Z
</commit_message>
<xml_diff>
--- a/data/coveragex/coveragex_latest.xlsx
+++ b/data/coveragex/coveragex_latest.xlsx
@@ -32242,14 +32242,14 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Auto-refreshed by GitHub Actions at 2026-10-29T17:28:08Z. Re-download from the published URL to get the latest.</t>
+          <t>Auto-refreshed by GitHub Actions at 2026-10-30T17:03:32Z. Re-download from the published URL to get the latest.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Last refreshed: 2026-10-29T17:28:08Z</t>
+          <t>Last refreshed: 2026-10-30T17:03:32Z</t>
         </is>
       </c>
     </row>
@@ -32317,7 +32317,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.99</v>
+        <v>5.05</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -32341,12 +32341,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -32387,12 +32387,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -32409,7 +32409,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -32433,12 +32433,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -32484,7 +32484,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -32530,7 +32530,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -32576,7 +32576,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -32622,7 +32622,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -32668,7 +32668,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -32714,7 +32714,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -32760,7 +32760,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-10-29T17:28:08Z</t>
+          <t>2026-10-30T17:03:32Z</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -32926,7 +32926,7 @@
         <v>0.556</v>
       </c>
       <c r="L18" t="n">
-        <v>291.2749938964844</v>
+        <v>293.2000122070312</v>
       </c>
     </row>
     <row r="19">
@@ -32970,7 +32970,7 @@
         <v>1.109</v>
       </c>
       <c r="L19" t="n">
-        <v>39.70000076293945</v>
+        <v>38.34999847412109</v>
       </c>
     </row>
     <row r="20">
@@ -33014,7 +33014,7 @@
         <v>1.184</v>
       </c>
       <c r="L20" t="n">
-        <v>55.42499923706055</v>
+        <v>55.18999862670898</v>
       </c>
     </row>
     <row r="21">
@@ -33058,7 +33058,7 @@
         <v>1.358</v>
       </c>
       <c r="L21" t="n">
-        <v>564.1199951171875</v>
+        <v>471.6499938964844</v>
       </c>
     </row>
     <row r="22">
@@ -33102,7 +33102,7 @@
         <v>1.05</v>
       </c>
       <c r="L22" t="n">
-        <v>208.7449951171875</v>
+        <v>203.8600006103516</v>
       </c>
     </row>
     <row r="23"/>

</xml_diff>